<commit_message>
fixed up image names
</commit_message>
<xml_diff>
--- a/DesignDocs/Rules.xlsx
+++ b/DesignDocs/Rules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A956972-1047-45E1-97F9-05FED5B76830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{06E26CB1-1E09-4BCD-A7B7-7B7D3A3606D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -407,25 +407,6 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='r2.2.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Other Counters&lt;LineBreak/&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;r0.0 They&amp;apos;ve Invaded Pleasantville&lt;/Bold&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-&lt;Bold&gt;Pleasantville&lt;/Bold&gt; minigame is a two-player game of a secret invasion by space aliens. One player, the Alien player, moves the Alien controlled and uncontrolled pieces, and the other player, the Town player, moves the Town-controlled pieces. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-There are 12 game-turns in this game. In any given turn, playing pieces representing various townspeople will be moved across the mapboard, which is a map of Pleasantville.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r1.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; How to Win&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r2.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Map and Counters&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r3.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Preparations for Play&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r4.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Sequence of Play&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r5.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Control&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r6.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Movement&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r7.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Conversation and Influence (Town player only)&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r8.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Combat&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r9.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Alien Take-Over And Observation
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Additional Rules can be viewed by selecting the &lt;Bold&gt;Help | Show Rules...&lt;/Bold&gt; menu.</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;r1.0 How to Win&lt;/Bold&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 The Alien player tries to keep the whereabouts of the Alien controlled townspeople a secret, while they 'take-over' more unsuspecting townspeople making them "zombies" and build up strength for the final showdown with the Town player. 
@@ -785,6 +766,25 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='Influence Modifiers' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table. 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 For example, if the Minister (influence factor=20) tries to influence the Supermarket Manager (influence factor=10), the ratio is 20 to 10 which simplifies to 2 to 1. All fractions are rounded down, so a 20 to 11 ratio reduces to 3-2 and not 2-1.</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;r0.0 Introduction&lt;/Bold&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+&lt;Bold&gt;They&amp;apos;ve Invaded Pleasantville&lt;/Bold&gt; minigame is a two-player game of a secret invasion by space aliens. One player, the Alien player, moves the Alien controlled and uncontrolled pieces, and the other player, the Town player, moves the Town-controlled pieces. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+There are 12 game-turns in this game. In any given turn, playing pieces representing various townspeople will be moved across the mapboard, which is a map of Pleasantville.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r1.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; How to Win&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r2.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Map and Counters&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r3.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Preparations for Play&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r4.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Sequence of Play&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r5.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Control&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r6.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Movement&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r7.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Conversation and Influence (Town player only)&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r8.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Combat&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r9.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Alien Take-Over And Observation
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Additional Rules can be viewed by selecting the &lt;Bold&gt;Help | Show Rules...&lt;/Bold&gt; menu.</t>
   </si>
 </sst>
 </file>
@@ -1166,7 +1166,7 @@
         <v>25</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>77</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -1174,7 +1174,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1190,7 +1190,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="270" x14ac:dyDescent="0.25">
@@ -1206,7 +1206,7 @@
         <v>26</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1214,7 +1214,7 @@
         <v>27</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1222,7 +1222,7 @@
         <v>28</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1230,7 +1230,7 @@
         <v>29</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1238,7 +1238,7 @@
         <v>30</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1246,7 +1246,7 @@
         <v>31</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1262,7 +1262,7 @@
         <v>32</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -1278,7 +1278,7 @@
         <v>34</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1286,7 +1286,7 @@
         <v>35</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1294,7 +1294,7 @@
         <v>36</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -1302,7 +1302,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1310,7 +1310,7 @@
         <v>13</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1326,7 +1326,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -1366,7 +1366,7 @@
         <v>12</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1374,7 +1374,7 @@
         <v>37</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1382,7 +1382,7 @@
         <v>38</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -1390,7 +1390,7 @@
         <v>39</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="270" x14ac:dyDescent="0.25">
@@ -1398,7 +1398,7 @@
         <v>40</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1406,7 +1406,7 @@
         <v>41</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1414,7 +1414,7 @@
         <v>2</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -1422,7 +1422,7 @@
         <v>3</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="210" x14ac:dyDescent="0.25">
@@ -1430,7 +1430,7 @@
         <v>4</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1438,7 +1438,7 @@
         <v>43</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1446,7 +1446,7 @@
         <v>44</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1462,7 +1462,7 @@
         <v>46</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -1502,7 +1502,7 @@
         <v>18</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -1518,7 +1518,7 @@
         <v>50</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1534,7 +1534,7 @@
         <v>21</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -1547,15 +1547,15 @@
     </row>
     <row r="49" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>72</v>
@@ -1563,7 +1563,7 @@
     </row>
     <row r="51" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>73</v>
@@ -1582,7 +1582,7 @@
         <v>23</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1598,7 +1598,7 @@
         <v>55</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -1606,7 +1606,7 @@
         <v>24</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -1614,7 +1614,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="120" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
changes to support initial welcome screen
</commit_message>
<xml_diff>
--- a/DesignDocs/Rules.xlsx
+++ b/DesignDocs/Rules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{06E26CB1-1E09-4BCD-A7B7-7B7D3A3606D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{89E3D4E8-C70F-4F2A-9470-8987315B632F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="1" r:id="rId1"/>
@@ -429,12 +429,6 @@
                             &lt;InlineUIContainer&gt;&lt;Image Name='Lawyer1'  Height='200' Width='200'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;r2.2.2 Counters - Starting Location&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-This letter on upper right of counter shows where the counter is placed on the map at the start of the game. For example, the Lawyer starts at building spot J, i.e., the Lawyer's Office.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                            &lt;InlineUIContainer&gt;&lt;Image Name='Lawyer2'  Height='200' Width='200'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;r2.1 Mapboard&lt;/Bold&gt;
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 The game map represents the main area of the town of Pleasantville. It has been divided into irregularly-shaped spaces for movement purposes. 
@@ -785,6 +779,14 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='r9.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Alien Take-Over And Observation
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Additional Rules can be viewed by selecting the &lt;Bold&gt;Help | Show Rules...&lt;/Bold&gt; menu.</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;r2.2.2 Counters - Starting Location&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+This letter on upper right of counter shows where the counter is placed on the map at the start of the game. For example, the Lawyer starts at building spot J, i.e., the Lawyer's Office.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Per &lt;InlineUIContainer&gt;&lt;Button Content='r3.4' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;, if a building has more than one space in it, the counter is placed randomly in one of the spaces. However, only one counter may be placed in each space.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                            &lt;InlineUIContainer&gt;&lt;Image Name='Lawyer2'  Height='200' Width='200'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -1166,7 +1168,7 @@
         <v>25</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -1190,7 +1192,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="270" x14ac:dyDescent="0.25">
@@ -1209,12 +1211,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1222,7 +1224,7 @@
         <v>28</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1230,7 +1232,7 @@
         <v>29</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1238,7 +1240,7 @@
         <v>30</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1246,7 +1248,7 @@
         <v>31</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1262,7 +1264,7 @@
         <v>32</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -1278,7 +1280,7 @@
         <v>34</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1286,7 +1288,7 @@
         <v>35</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1294,7 +1296,7 @@
         <v>36</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -1302,7 +1304,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1310,7 +1312,7 @@
         <v>13</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1326,7 +1328,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -1366,7 +1368,7 @@
         <v>12</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1374,7 +1376,7 @@
         <v>37</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1382,7 +1384,7 @@
         <v>38</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -1390,7 +1392,7 @@
         <v>39</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="270" x14ac:dyDescent="0.25">
@@ -1398,7 +1400,7 @@
         <v>40</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1406,7 +1408,7 @@
         <v>41</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1414,7 +1416,7 @@
         <v>2</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -1422,7 +1424,7 @@
         <v>3</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="210" x14ac:dyDescent="0.25">
@@ -1430,7 +1432,7 @@
         <v>4</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1438,7 +1440,7 @@
         <v>43</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1446,7 +1448,7 @@
         <v>44</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1462,7 +1464,7 @@
         <v>46</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -1502,7 +1504,7 @@
         <v>18</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -1518,7 +1520,7 @@
         <v>50</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1534,7 +1536,7 @@
         <v>21</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -1547,15 +1549,15 @@
     </row>
     <row r="49" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>72</v>
@@ -1563,7 +1565,7 @@
     </row>
     <row r="51" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>73</v>
@@ -1582,7 +1584,7 @@
         <v>23</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1598,7 +1600,7 @@
         <v>55</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -1606,7 +1608,7 @@
         <v>24</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -1614,7 +1616,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="120" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
unit test Territory utilitie functions
</commit_message>
<xml_diff>
--- a/DesignDocs/Rules.xlsx
+++ b/DesignDocs/Rules.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\Documents\HereWeGo\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38242897-86A6-4CDB-B1FA-BEDB5192FFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{96EC9185-0D3E-4AE8-9EBF-40461B9F0501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-27240" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>

<commit_message>
combat fix and takeover fix
</commit_message>
<xml_diff>
--- a/DesignDocs/Rules.xlsx
+++ b/DesignDocs/Rules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BADD01F-82CC-4B7D-9B8C-E634BBC83D99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D2DE120-E856-4DD7-9026-C720276276D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="90" windowWidth="29040" windowHeight="15510" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="1" r:id="rId1"/>
@@ -332,13 +332,6 @@
 Only four choices may be made per interrogation, and each Alien controlled counter may only be interrogated once. </t>
   </si>
   <si>
-    <t>&lt;Bold&gt;r9.0 Alien Take-Over And Observation&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-During this phase, the Alien player may 'take-over' uncontrolled townspeople, thus bringing them under Alien control. This is handled secretly so the Town player does know know which counters are Alien controlled.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r9.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Take-Over&lt;LineBreak/&gt;
-&lt;InlineUIContainer&gt;&lt;Button Content='r9.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Observation&lt;LineBreak/&gt;</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;r9.1.1 Take-over Example&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
 At the beginning of this phase, the Alien player finds three spaces on the board that are holding more than one counter. However, the counters in one space are Town controlled, so the Alien player cannot affect them. 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
@@ -786,6 +779,13 @@
 Successfully removing the implant causes the victim to come under control of the Town player. If an implant is removed intact, it can be carried as evidence. Such evidence adds +1 to the influence roll when the townsperson carrying the implant tries to influence another townsperson per &lt;InlineUIContainer&gt;&lt;Button Content='r7.2.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 As only Alien controlled counters may be interrogated, it is wise to interrogate per &lt;InlineUIContainer&gt;&lt;Button Content='r8.7.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  before attempting to remove an implant. Removing the implant generates an electric shock which erases all memory of the Alien HQ from the victim's memory, a unique safegard which is built into the implant's circuits.</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;r9.0 Alien Take-Over And Observation&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+During this phase, the Alien player may 'take-over' uncontrolled townspeople or stunned controlled Town pieces (but not unconscious), thus bringing them under Alien control. This is handled secretly so the Town player does know know which counters are Alien controlled.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r9.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Take-Over&lt;LineBreak/&gt;
+&lt;InlineUIContainer&gt;&lt;Button Content='r9.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Observation&lt;LineBreak/&gt;</t>
   </si>
 </sst>
 </file>
@@ -1167,7 +1167,7 @@
         <v>25</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -1175,7 +1175,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1191,7 +1191,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="270" x14ac:dyDescent="0.25">
@@ -1199,7 +1199,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1207,7 +1207,7 @@
         <v>26</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1215,7 +1215,7 @@
         <v>27</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1223,7 +1223,7 @@
         <v>28</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1231,7 +1231,7 @@
         <v>29</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1239,7 +1239,7 @@
         <v>30</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1247,7 +1247,7 @@
         <v>31</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1263,7 +1263,7 @@
         <v>32</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -1279,7 +1279,7 @@
         <v>34</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1287,7 +1287,7 @@
         <v>35</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1295,7 +1295,7 @@
         <v>36</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -1303,7 +1303,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1311,7 +1311,7 @@
         <v>13</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1327,7 +1327,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -1367,7 +1367,7 @@
         <v>12</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1375,7 +1375,7 @@
         <v>37</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1383,7 +1383,7 @@
         <v>38</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -1391,7 +1391,7 @@
         <v>39</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="270" x14ac:dyDescent="0.25">
@@ -1399,7 +1399,7 @@
         <v>40</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1407,7 +1407,7 @@
         <v>41</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1415,7 +1415,7 @@
         <v>2</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -1423,7 +1423,7 @@
         <v>3</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="210" x14ac:dyDescent="0.25">
@@ -1431,7 +1431,7 @@
         <v>4</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1439,7 +1439,7 @@
         <v>43</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1447,7 +1447,7 @@
         <v>44</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1463,7 +1463,7 @@
         <v>46</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -1487,7 +1487,7 @@
         <v>16</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1503,7 +1503,7 @@
         <v>18</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="132.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1519,7 +1519,7 @@
         <v>50</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1535,7 +1535,7 @@
         <v>21</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -1543,20 +1543,20 @@
         <v>52</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>69</v>
@@ -1564,18 +1564,18 @@
     </row>
     <row r="51" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>70</v>
+        <v>115</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1583,7 +1583,7 @@
         <v>23</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1591,7 +1591,7 @@
         <v>53</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1599,7 +1599,7 @@
         <v>54</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -1607,7 +1607,7 @@
         <v>24</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -1615,7 +1615,7 @@
         <v>55</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1623,7 +1623,7 @@
         <v>56</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
working retreating stunned counters
</commit_message>
<xml_diff>
--- a/DesignDocs/Rules.xlsx
+++ b/DesignDocs/Rules.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D2DE120-E856-4DD7-9026-C720276276D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{20CE4A1D-8F7A-4B91-AD85-60DFE34AC853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -614,19 +614,6 @@
 Note that the Welder is the Attacker even though the Wife started the combat.</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;r8.6 Combat - Results&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-There are four results that can occur from combat:&lt;LineBreak/&gt;&lt;LineBreak/&gt;
--- Attacker Flees (AF): Each counter of the Attacker must flee using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. If the counter is already in the building, roll again until a different target building is determined. The Alien Sub-Commander cannot flee and instead defeated. Should the Town Player defeat the Sub-Commander, the game is automatically ended with a Town player victory.
-&lt;LineBreak/&gt;.&lt;LineBreak/&gt;
--- Defender Flees (DF): Same mechanics as Attacker flees but for Defender.
-&lt;LineBreak/&gt;.&lt;LineBreak/&gt;
--- Attacker Wins (A): Consult the appropriate table: 
- &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table or  
- &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table. The dice are rolled for each individual counter of the defeated force, and the results are applied immediately.  Should the Town Player defeat the Sub-Commander, the game is automatically ended with a Town player victory!.
-&lt;LineBreak/&gt;.&lt;LineBreak/&gt;
--- Defender Wins (D): Same mechanics as Attacker Wins but for Defender.</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;r9.1.2 Take-over Restrictions&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Take-over can occur in any space on the board. One of the two counters must be already Alien controlled. 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
@@ -786,6 +773,19 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Content='r9.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Take-Over&lt;LineBreak/&gt;
 &lt;InlineUIContainer&gt;&lt;Button Content='r9.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Observation&lt;LineBreak/&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;r8.6 Combat - Results&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+There are four results that can occur from combat:&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+-- Attacker Flees (AF): Each counter of the Attacker must flee using Random Movement per &lt;InlineUIContainer&gt;&lt;Button Content='r6.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. If the counter is already in the building, roll again until a different target building is determined. The Alien Sub-Commander cannot flee and instead defeated. Should the Town Player defeat the Sub-Commander, the game is automatically ended with a Town player victory.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+-- Defender Flees (DF): Same mechanics as Attacker flees but for Defender.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+-- Attacker Wins (A): Consult the appropriate table: 
+ &lt;InlineUIContainer&gt;&lt;Button Content='Alien Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table or  
+ &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table. The dice are rolled for each individual counter of the defeated force, and the results are applied immediately.  Should the Town Player defeat the Sub-Commander, the game is automatically ended with a Town player victory!.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+-- Defender Wins (D): Same mechanics as Attacker Wins but for Defender.</t>
   </si>
 </sst>
 </file>
@@ -1167,7 +1167,7 @@
         <v>25</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -1215,7 +1215,7 @@
         <v>27</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1279,7 +1279,7 @@
         <v>34</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1367,7 +1367,7 @@
         <v>12</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1391,7 +1391,7 @@
         <v>39</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="270" x14ac:dyDescent="0.25">
@@ -1407,7 +1407,7 @@
         <v>41</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1439,7 +1439,7 @@
         <v>43</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1463,7 +1463,7 @@
         <v>46</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -1487,7 +1487,7 @@
         <v>16</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1535,7 +1535,7 @@
         <v>21</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -1543,7 +1543,7 @@
         <v>52</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1567,7 +1567,7 @@
         <v>86</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1575,7 +1575,7 @@
         <v>22</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1583,7 +1583,7 @@
         <v>23</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1599,7 +1599,7 @@
         <v>54</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -1607,7 +1607,7 @@
         <v>24</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -1623,7 +1623,7 @@
         <v>56</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix teacher gif. Fix Rule Text. Show blank roll if observer is alien. All units must participate in combat.
</commit_message>
<xml_diff>
--- a/DesignDocs/Rules.xlsx
+++ b/DesignDocs/Rules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\TheyveInvadedPleasantville\DesignDocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstewa01\source\repos\happysulla\TheyveInvadedPleasantville\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{20CE4A1D-8F7A-4B91-AD85-60DFE34AC853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{091A0E54-08F3-4336-82B2-3516D8101600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
+    <workbookView xWindow="-120" yWindow="90" windowWidth="29040" windowHeight="15510" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="1" r:id="rId1"/>
@@ -189,15 +189,6 @@
     <t>r8.4</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;Bold&gt;r8.1 Combat - General Rules&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Combat takes place only between counters sharing the same space. It is not permitted to attack a counter in an adjacent space.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-All combat is voluntary. Neither player is forced to start combat. Thus, combat takes place only when at least one player desires it.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Either player may start combat as desired. Combat for each space is resolved separately and individually. There is no way combat in one are will affect combat in another area. Each counter may only be involved in one combat per turn.
-</t>
-  </si>
-  <si>
     <t>r8.7</t>
   </si>
   <si>
@@ -786,6 +777,15 @@
  &lt;InlineUIContainer&gt;&lt;Button Content='Town Loss' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table. The dice are rolled for each individual counter of the defeated force, and the results are applied immediately.  Should the Town Player defeat the Sub-Commander, the game is automatically ended with a Town player victory!.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 -- Defender Wins (D): Same mechanics as Attacker Wins but for Defender.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;Bold&gt;r8.1 Combat - General Rules&lt;/Bold&gt;&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Combat takes place only between counters sharing the same space. It is not permitted to attack a counter in an adjacent space.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+All combat is voluntary. Neither player is forced to start combat. Thus, combat takes place only when at least one player desires it.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Either player may start combat as desired. Combat for each space is resolved separately and individually. Combat in one area will not affect combat in another area. Each counter may only be involved in one combat per turn.
+</t>
   </si>
 </sst>
 </file>
@@ -1167,7 +1167,7 @@
         <v>25</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="240" x14ac:dyDescent="0.25">
@@ -1175,7 +1175,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1183,7 +1183,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -1191,7 +1191,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="270" x14ac:dyDescent="0.25">
@@ -1199,7 +1199,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1207,7 +1207,7 @@
         <v>26</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1215,7 +1215,7 @@
         <v>27</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1223,7 +1223,7 @@
         <v>28</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1231,7 +1231,7 @@
         <v>29</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1239,7 +1239,7 @@
         <v>30</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1247,7 +1247,7 @@
         <v>31</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1255,7 +1255,7 @@
         <v>7</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1263,7 +1263,7 @@
         <v>32</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="45" x14ac:dyDescent="0.25">
@@ -1271,7 +1271,7 @@
         <v>33</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1279,7 +1279,7 @@
         <v>34</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1287,7 +1287,7 @@
         <v>35</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1295,7 +1295,7 @@
         <v>36</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -1303,7 +1303,7 @@
         <v>1</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1311,7 +1311,7 @@
         <v>13</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1319,7 +1319,7 @@
         <v>14</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1327,7 +1327,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -1335,7 +1335,7 @@
         <v>42</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="210" x14ac:dyDescent="0.25">
@@ -1343,7 +1343,7 @@
         <v>9</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1351,7 +1351,7 @@
         <v>10</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -1359,7 +1359,7 @@
         <v>11</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="195" x14ac:dyDescent="0.25">
@@ -1367,7 +1367,7 @@
         <v>12</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1375,7 +1375,7 @@
         <v>37</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1383,7 +1383,7 @@
         <v>38</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -1391,7 +1391,7 @@
         <v>39</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="270" x14ac:dyDescent="0.25">
@@ -1399,7 +1399,7 @@
         <v>40</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1407,7 +1407,7 @@
         <v>41</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1415,7 +1415,7 @@
         <v>2</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -1423,7 +1423,7 @@
         <v>3</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="210" x14ac:dyDescent="0.25">
@@ -1431,7 +1431,7 @@
         <v>4</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1439,7 +1439,7 @@
         <v>43</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1447,7 +1447,7 @@
         <v>44</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -1455,7 +1455,7 @@
         <v>45</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -1463,7 +1463,7 @@
         <v>46</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -1479,7 +1479,7 @@
         <v>48</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -1487,7 +1487,7 @@
         <v>16</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -1495,7 +1495,7 @@
         <v>17</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>51</v>
+        <v>115</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="225" x14ac:dyDescent="0.25">
@@ -1503,7 +1503,7 @@
         <v>18</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="132.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1511,7 +1511,7 @@
         <v>19</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1519,7 +1519,7 @@
         <v>50</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1527,7 +1527,7 @@
         <v>20</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="210" x14ac:dyDescent="0.25">
@@ -1535,39 +1535,39 @@
         <v>21</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -1575,7 +1575,7 @@
         <v>22</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -1583,23 +1583,23 @@
         <v>23</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -1607,23 +1607,23 @@
         <v>24</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="240" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>